<commit_message>
fix: update KBSV PROD config and JWE encryption
</commit_message>
<xml_diff>
--- a/data/CPI_VNM.xlsx
+++ b/data/CPI_VNM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0. Luu_Thu Huyen\Nam 2026\CPI\Tháng 5.2026\0. GỬI NGÂN CÔNG BỐ THÁNG 5.2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0. Luu_Thu Huyen\Nam 2026\CPI\Tháng 6.2026\0. CÔNG BỐ THÁNG 6.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="238">
   <si>
     <t>DATA_DOMAIN</t>
   </si>
@@ -736,6 +736,9 @@
   </si>
   <si>
     <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
   </si>
 </sst>
 </file>
@@ -1258,7 +1261,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{44889A44-8645-4601-8977-B14930E482A0}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44889A44-8645-4601-8977-B14930E482A0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9117,6 +9120,9 @@
       <c r="M11" s="61" t="s">
         <v>236</v>
       </c>
+      <c r="N11" s="61" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="12" spans="1:16 15819:15826" s="8" customFormat="1">
       <c r="A12" s="20"/>
@@ -9170,6 +9176,9 @@
       </c>
       <c r="M13" s="52">
         <v>108.04437502096535</v>
+      </c>
+      <c r="N13" s="52">
+        <v>107.62753982213445</v>
       </c>
       <c r="P13" s="55"/>
       <c r="WJK13" s="4"/>
@@ -9217,6 +9226,9 @@
       <c r="M14" s="52">
         <v>107.29822231667669</v>
       </c>
+      <c r="N14" s="52">
+        <v>107.22064570194172</v>
+      </c>
       <c r="P14" s="55"/>
       <c r="WJK14" s="4"/>
       <c r="WJL14" s="4"/>
@@ -9263,6 +9275,9 @@
       <c r="M15" s="52">
         <v>102.37330204842654</v>
       </c>
+      <c r="N15" s="52">
+        <v>101.57458554584473</v>
+      </c>
       <c r="P15" s="55"/>
       <c r="WJK15" s="4"/>
       <c r="WJL15" s="4"/>
@@ -9309,6 +9324,9 @@
       <c r="M16" s="52">
         <v>107.04559292619518</v>
       </c>
+      <c r="N16" s="52">
+        <v>106.98714603245749</v>
+      </c>
       <c r="P16" s="55"/>
       <c r="WJK16" s="4"/>
       <c r="WJL16" s="4"/>
@@ -9355,6 +9373,9 @@
       <c r="M17" s="52">
         <v>110.17452096408124</v>
       </c>
+      <c r="N17" s="52">
+        <v>110.39564122765614</v>
+      </c>
       <c r="P17" s="55"/>
       <c r="WJK17" s="4"/>
       <c r="WJL17" s="4"/>
@@ -9401,6 +9422,9 @@
       <c r="M18" s="52">
         <v>105.57158948997565</v>
       </c>
+      <c r="N18" s="52">
+        <v>105.70545426544894</v>
+      </c>
       <c r="P18" s="55"/>
       <c r="WJK18" s="4"/>
       <c r="WJL18" s="4"/>
@@ -9447,6 +9471,9 @@
       <c r="M19" s="52">
         <v>103.44137658207032</v>
       </c>
+      <c r="N19" s="52">
+        <v>103.35334797059899</v>
+      </c>
       <c r="P19" s="55"/>
       <c r="WJK19" s="4"/>
       <c r="WJL19" s="4"/>
@@ -9493,6 +9520,9 @@
       <c r="M20" s="52">
         <v>112.61352511455581</v>
       </c>
+      <c r="N20" s="52">
+        <v>113.13256085180879</v>
+      </c>
       <c r="P20" s="55"/>
       <c r="WJK20" s="4"/>
       <c r="WJL20" s="4"/>
@@ -9539,6 +9569,9 @@
       <c r="M21" s="52">
         <v>104.78067546107447</v>
       </c>
+      <c r="N21" s="52">
+        <v>104.96089822286751</v>
+      </c>
       <c r="P21" s="55"/>
       <c r="WJK21" s="4"/>
       <c r="WJL21" s="4"/>
@@ -9585,6 +9618,9 @@
       <c r="M22" s="52">
         <v>107.31404901044777</v>
       </c>
+      <c r="N22" s="52">
+        <v>107.34849682018013</v>
+      </c>
       <c r="P22" s="55"/>
       <c r="WJK22" s="4"/>
       <c r="WJL22" s="4"/>
@@ -9631,6 +9667,9 @@
       <c r="M23" s="52">
         <v>109.41394939631034</v>
       </c>
+      <c r="N23" s="52">
+        <v>109.41121404757543</v>
+      </c>
       <c r="P23" s="55"/>
       <c r="WJK23" s="4"/>
       <c r="WJL23" s="4"/>
@@ -9677,6 +9716,9 @@
       <c r="M24" s="52">
         <v>106.69170643352061</v>
       </c>
+      <c r="N24" s="52">
+        <v>101.5223865651101</v>
+      </c>
       <c r="P24" s="55"/>
       <c r="WJK24" s="4"/>
       <c r="WJL24" s="4"/>
@@ -9723,6 +9765,9 @@
       <c r="M25" s="52">
         <v>100.4687287323332</v>
       </c>
+      <c r="N25" s="52">
+        <v>100.51132747331572</v>
+      </c>
       <c r="P25" s="55"/>
       <c r="WJK25" s="4"/>
       <c r="WJL25" s="4"/>
@@ -9769,6 +9814,9 @@
       <c r="M26" s="52">
         <v>111.35782349271605</v>
       </c>
+      <c r="N26" s="52">
+        <v>111.37274544106407</v>
+      </c>
       <c r="P26" s="55"/>
       <c r="WJN26" s="4"/>
       <c r="WJO26" s="4"/>
@@ -9815,6 +9863,9 @@
       <c r="M27" s="52">
         <v>112.53887591853609</v>
       </c>
+      <c r="N27" s="52">
+        <v>112.60831240497782</v>
+      </c>
       <c r="P27" s="55"/>
       <c r="WJN27" s="4"/>
       <c r="WJO27" s="4"/>
@@ -9861,6 +9912,9 @@
       <c r="M28" s="52">
         <v>103.78890616578722</v>
       </c>
+      <c r="N28" s="52">
+        <v>104.47640388022941</v>
+      </c>
       <c r="P28" s="55"/>
       <c r="WJK28" s="4"/>
       <c r="WJL28" s="4"/>
@@ -9907,6 +9961,9 @@
       <c r="M29" s="52">
         <v>109.10681458075479</v>
       </c>
+      <c r="N29" s="52">
+        <v>109.04582387140415</v>
+      </c>
       <c r="P29" s="55"/>
       <c r="WJK29" s="4"/>
       <c r="WJL29" s="4"/>
@@ -9967,6 +10024,9 @@
       <c r="M31" s="52">
         <v>100</v>
       </c>
+      <c r="N31" s="52">
+        <v>100</v>
+      </c>
     </row>
     <row r="32" spans="1:16 15819:15826">
       <c r="A32" s="16" t="s">
@@ -10008,8 +10068,11 @@
       <c r="M32" s="52">
         <v>35.823212593699999</v>
       </c>
-    </row>
-    <row r="33" spans="1:13 15825:15826">
+      <c r="N32" s="52">
+        <v>35.823212593699999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14 15825:15826">
       <c r="A33" s="16" t="s">
         <v>104</v>
       </c>
@@ -10049,8 +10112,11 @@
       <c r="M33" s="52">
         <v>4.1456756961000005</v>
       </c>
-    </row>
-    <row r="34" spans="1:13 15825:15826">
+      <c r="N33" s="52">
+        <v>4.1456756961000005</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14 15825:15826">
       <c r="A34" s="16" t="s">
         <v>122</v>
       </c>
@@ -10090,8 +10156,11 @@
       <c r="M34" s="52">
         <v>22.323992676</v>
       </c>
-    </row>
-    <row r="35" spans="1:13 15825:15826">
+      <c r="N34" s="52">
+        <v>22.323992676</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14 15825:15826">
       <c r="A35" s="60" t="s">
         <v>170</v>
       </c>
@@ -10131,8 +10200,11 @@
       <c r="M35" s="52">
         <v>9.3535442217</v>
       </c>
-    </row>
-    <row r="36" spans="1:13 15825:15826">
+      <c r="N35" s="52">
+        <v>9.3535442217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14 15825:15826">
       <c r="A36" s="16" t="s">
         <v>105</v>
       </c>
@@ -10172,8 +10244,11 @@
       <c r="M36" s="52">
         <v>1.7513242057</v>
       </c>
-    </row>
-    <row r="37" spans="1:13 15825:15826">
+      <c r="N36" s="52">
+        <v>1.7513242057</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14 15825:15826">
       <c r="A37" s="16" t="s">
         <v>106</v>
       </c>
@@ -10213,8 +10288,11 @@
       <c r="M37" s="52">
         <v>3.5220945052000001</v>
       </c>
-    </row>
-    <row r="38" spans="1:13 15825:15826" ht="45">
+      <c r="N37" s="52">
+        <v>3.5220945052000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14 15825:15826" ht="45">
       <c r="A38" s="16" t="s">
         <v>107</v>
       </c>
@@ -10254,8 +10332,11 @@
       <c r="M38" s="52">
         <v>22.697484706599997</v>
       </c>
-    </row>
-    <row r="39" spans="1:13 15825:15826">
+      <c r="N38" s="52">
+        <v>22.697484706599997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14 15825:15826">
       <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
@@ -10295,8 +10376,11 @@
       <c r="M39" s="52">
         <v>5.1430623014000005</v>
       </c>
-    </row>
-    <row r="40" spans="1:13 15825:15826">
+      <c r="N39" s="52">
+        <v>5.1430623014000005</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14 15825:15826">
       <c r="A40" s="16" t="s">
         <v>109</v>
       </c>
@@ -10336,8 +10420,11 @@
       <c r="M40" s="52">
         <v>4.6611529854999993</v>
       </c>
-    </row>
-    <row r="41" spans="1:13 15825:15826">
+      <c r="N40" s="52">
+        <v>4.6611529854999993</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14 15825:15826">
       <c r="A41" s="16" t="s">
         <v>110</v>
       </c>
@@ -10377,8 +10464,11 @@
       <c r="M41" s="52">
         <v>9.9795999999999996</v>
       </c>
-    </row>
-    <row r="42" spans="1:13 15825:15826" ht="30">
+      <c r="N41" s="52">
+        <v>9.9795999999999996</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14 15825:15826" ht="30">
       <c r="A42" s="16" t="s">
         <v>111</v>
       </c>
@@ -10418,8 +10508,11 @@
       <c r="M42" s="52">
         <v>3.7356383262000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:13 15825:15826">
+      <c r="N42" s="52">
+        <v>3.7356383262000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14 15825:15826">
       <c r="A43" s="16" t="s">
         <v>112</v>
       </c>
@@ -10459,8 +10552,11 @@
       <c r="M43" s="52">
         <v>5.9637911495000004</v>
       </c>
-    </row>
-    <row r="44" spans="1:13 15825:15826" ht="30">
+      <c r="N43" s="52">
+        <v>5.9637911495000004</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14 15825:15826" ht="30">
       <c r="A44" s="16" t="s">
         <v>113</v>
       </c>
@@ -10500,8 +10596,11 @@
       <c r="M44" s="52">
         <v>3.1426392262</v>
       </c>
-    </row>
-    <row r="45" spans="1:13 15825:15826" ht="30">
+      <c r="N44" s="52">
+        <v>3.1426392262</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14 15825:15826" ht="30">
       <c r="A45" s="16" t="s">
         <v>114</v>
       </c>
@@ -10541,8 +10640,11 @@
       <c r="M45" s="52">
         <v>3.58</v>
       </c>
-    </row>
-    <row r="46" spans="1:13 15825:15826" s="8" customFormat="1">
+      <c r="N45" s="52">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14 15825:15826" s="8" customFormat="1">
       <c r="A46" s="20"/>
       <c r="B46" s="21" t="s">
         <v>115</v>
@@ -10555,7 +10657,7 @@
       <c r="WJQ46" s="23"/>
       <c r="WJR46" s="23"/>
     </row>
-    <row r="47" spans="1:13 15825:15826">
+    <row r="47" spans="1:14 15825:15826">
       <c r="A47" s="58" t="s">
         <v>120</v>
       </c>
@@ -10594,6 +10696,9 @@
       </c>
       <c r="M47" s="52">
         <v>4.6678117720838852</v>
+      </c>
+      <c r="N47" s="52">
+        <v>4.4957618993496817</v>
       </c>
     </row>
   </sheetData>

</xml_diff>